<commit_message>
freeze post refinement evidence and browser checks
Preserve the initial after set as superseded and freeze the single cleanup confirmation for round two. Record passing frontend checks and four native-browser cases, with scope limits and audited detector findings.

Co-Authored-By: GPT-6.1-Sol <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/docs/ui-post-eight/KyPost-Council.xlsx
+++ b/docs/ui-post-eight/KyPost-Council.xlsx
@@ -5077,6 +5077,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
document post reader controls and review checkpoint
Keep operator feature summaries aligned with the reader controls and expose the PR link in the Council workbook while round two and current-head CI run.

Co-Authored-By: GPT-6.1-Sol <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/docs/ui-post-eight/KyPost-Council.xlsx
+++ b/docs/ui-post-eight/KyPost-Council.xlsx
@@ -7,6 +7,7 @@
     <sheet name="Progression" sheetId="3" r:id="rId3"/>
     <sheet name="Spreads" sheetId="4" r:id="rId4"/>
     <sheet name="Notes" sheetId="5" r:id="rId5"/>
+    <sheet name="Delivery" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -11385,4 +11386,107 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">repository</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Busnes-app/KyPost-Server</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">url</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/Busnes-app/KyPost-Server/pull/489</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">branch</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/post-eight</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui_source</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">50bbbff5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evidence</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b6852d8f</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">status</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">open; whole-repository current-head CI/security and R2 primary scores pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">merge_deploy_authorized</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
freeze kypost control consistency evidence
Record the current 32-image set, focused browser checks and corrected Opus-only progression rule. Preserve prior reports and explicitly supersede the earlier pooled acceptance.
</commit_message>
<xml_diff>
--- a/docs/ui-post-eight/KyPost-Council.xlsx
+++ b/docs/ui-post-eight/KyPost-Council.xlsx
@@ -9908,17 +9908,17 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Combined exact</t>
+          <t xml:space="preserve">Historical combined exact (not gate)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rounded</t>
+          <t xml:space="preserve">Opus rounded</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted</t>
+          <t xml:space="preserve">Accepted by current rule</t>
         </is>
       </c>
     </row>
@@ -9945,7 +9945,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.2</t>
+          <t xml:space="preserve">6.8</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -9977,12 +9977,44 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8.0</t>
+          <t xml:space="preserve">7.6</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">True</t>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
     </row>
@@ -22376,7 +22408,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same-set Claude/Sol quality mean, half-up to one decimal; &gt;=8.0 accepts. Brand is separate; raw scores/satisfaction retained.</t>
+          <t xml:space="preserve">Opus overall current-round quality mean, half-up to one decimal; &gt;=8.0 accepts. Sol is independent. Prior combined-score acceptance is superseded; historical reports are immutable. Brand is separate.</t>
         </is>
       </c>
     </row>
@@ -22455,7 +22487,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://github.com/Busnes-app/KyPost-Server/pull/489</t>
+          <t xml:space="preserve">Pending follow-up PR</t>
         </is>
       </c>
     </row>
@@ -22467,7 +22499,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ui/post-eight</t>
+          <t xml:space="preserve">ui/post-control-consistency</t>
         </is>
       </c>
     </row>
@@ -22479,7 +22511,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">50bbbff5</t>
+          <t xml:space="preserve">2ff40cc2394d1bab8cf14935ba6b219a5f28b8f1</t>
         </is>
       </c>
     </row>
@@ -22503,7 +22535,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">open; visual progression accepted8.0; whole-repository current-head CI/security pending</t>
+          <t xml:space="preserve">reopened under clarified Opus-only gate; round3 primary reviews pending</t>
         </is>
       </c>
     </row>
@@ -22527,7 +22559,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">2 complete,3pending</t>
         </is>
       </c>
     </row>
@@ -22539,7 +22571,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">513/64</t>
+          <t xml:space="preserve">513/64 (historical, not gate)</t>
         </is>
       </c>
     </row>
@@ -22551,7 +22583,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">8.0</t>
+          <t xml:space="preserve">8.0 (historical, not gate)</t>
         </is>
       </c>
     </row>
@@ -22563,7 +22595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">True</t>
+          <t xml:space="preserve">False</t>
         </is>
       </c>
     </row>
@@ -22576,6 +22608,30 @@
       <c r="B13" t="inlineStr">
         <is>
           <t xml:space="preserve">Unused; both primaries not independently satisfied</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">opus_rounded</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7.6; previous captured set</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">previous_pr</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/Busnes-app/KyPost-Server/pull/489</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
record unavailable gemini advisory without delaying progress
Preserve the quota response as an unavailable review with no score or findings. Keep the accepted Opus progression decision and export the final reviewer status.

Co-Authored-By: GPT-6.1-Sol <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/docs/ui-post-eight/KyPost-Council.xlsx
+++ b/docs/ui-post-eight/KyPost-Council.xlsx
@@ -44540,7 +44540,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"round": 4, "raw_reports": {"opus-round4.json": "fc9763aefe34753e8fa12601e85ec7f663b16d459c62c20bf16d43e53276c095", "opus-round4.md": "ad917b57e27b922c06751e988b7da8439c23fe93c22c4ed007e22c56ddbd15da", "sol-round4.json": "9e6ebf14198418c5b755dd6671f6ad33eae0ee14094092157b6b76b8830cceb8", "sol-round4.md": "df1a598f2bd5d6f23eecbc19a88f31fe8e4abed926115cf96bbc09e7c7530f90"}, "source_ui": "558761afa10560a5ba9522e6d7603dbf2a17ccfd", "frozen_evidence": "f53e76ced2506284b393baffbc3f181ba4549543", "membership": "Both report sets match all32 stage06 originals; hashes and exact weighted totals independently reproduced.", "progression": {"opus_exact": "1277/160", "opus_decimal": "7.98125", "opus_rounded": "8.0", "accepted": true, "sol_exact": "1369/160", "sol_decimal": "8.55625", "rule": "Opus current overall only, half-up to0.1. No pooling with Sol, brand or history."}, "independent_satisfaction": {"opus": {"satisfied": true, "genuinely_satisfied": true}, "sol": {"satisfied": true, "genuinely_satisfied": true}}, "spread_audit": {"dimensions_ge_2": 2, "entries": [{"file": "screenshots/kypost-06-after-contacts-mobile-dark.png", "dimension": "density_layout", "opus": 6, "sol": 8}, {"file": "screenshots/kypost-06-after-contacts-mobile-light.png", "dimension": "density_layout", "opus": 6, "sol": 8}], "inspection": "Parent re-opened both stage06 phone contacts originals individually at native resolution. Approximately137px rows split name, email and action text across different left edges; the search hint clips. Opus6 vsSol8 density is a valid judgment spread, retained unchanged. No broken view or progression veto.", "resolution": "Retain both raw vectors and findings; no averaged replacement or cosmetic round."}, "freeze_integrity": {"opus": "Verified persisted checks/opus-r4-freeze.json bytes against publisher hash. Quality vectors, observations, totals, brand vectors/observations/N/A exclusions all unchanged. Final brand records add mean_exact_fraction only (all32); raw full-vector digest therefore differs if derived metadata is included.", "opus_frozen_file_sha256": "8fe9a11f471f7fc4efe0557de120ad6313a26a5748472248ec4ee1ab1dc85a97", "sol": "Full files-array digest reproduces050708ca86dab5500f6bf13595fa14bf7ff4b006d6c08a40a6689ae66c8958e0."}, "drift": "Opus raw mean rises0.09375; Sol raw mean falls0.1. Both disclose variance on unchanged images. Never use variance-adjusted estimates as progression scores.", "remaining_findings": ["Phone contacts row density/alignment, clipped search hint and repeated count.", "Contact-editor photo helper placement and disclosure spacing.", "Phone bulk toolbar wrap; optional navigation-label consistency."], "limitations": ["Everyday-user initial views only; full behavior/roles/states/all named themes/assistive-tech/competitive gates remain untested.", "Opus live supplement uses a different browser/DPR and does not replace scored originals.", "Current-head whole-repository hostedCI and security review remain pending."], "gemini": "Advisory pending; launched only after both primaries genuinely satisfied. Acceptance is already decided.", "dox_pass": "Evidence records and existing exporter only. Owning AGENTS and parent indexes intentionally unchanged: ownership, structure and progression contracts are unchanged."}</t>
+          <t xml:space="preserve">{"round": 4, "raw_reports": {"opus-round4.json": "fc9763aefe34753e8fa12601e85ec7f663b16d459c62c20bf16d43e53276c095", "opus-round4.md": "ad917b57e27b922c06751e988b7da8439c23fe93c22c4ed007e22c56ddbd15da", "sol-round4.json": "9e6ebf14198418c5b755dd6671f6ad33eae0ee14094092157b6b76b8830cceb8", "sol-round4.md": "df1a598f2bd5d6f23eecbc19a88f31fe8e4abed926115cf96bbc09e7c7530f90"}, "source_ui": "558761afa10560a5ba9522e6d7603dbf2a17ccfd", "frozen_evidence": "f53e76ced2506284b393baffbc3f181ba4549543", "membership": "Both report sets match all32 stage06 originals; hashes and exact weighted totals independently reproduced.", "progression": {"opus_exact": "1277/160", "opus_decimal": "7.98125", "opus_rounded": "8.0", "accepted": true, "sol_exact": "1369/160", "sol_decimal": "8.55625", "rule": "Opus current overall only, half-up to0.1. No pooling with Sol, brand or history."}, "independent_satisfaction": {"opus": {"satisfied": true, "genuinely_satisfied": true}, "sol": {"satisfied": true, "genuinely_satisfied": true}}, "spread_audit": {"dimensions_ge_2": 2, "entries": [{"file": "screenshots/kypost-06-after-contacts-mobile-dark.png", "dimension": "density_layout", "opus": 6, "sol": 8}, {"file": "screenshots/kypost-06-after-contacts-mobile-light.png", "dimension": "density_layout", "opus": 6, "sol": 8}], "inspection": "Parent re-opened both stage06 phone contacts originals individually at native resolution. Approximately137px rows split name, email and action text across different left edges; the search hint clips. Opus6 vsSol8 density is a valid judgment spread, retained unchanged. No broken view or progression veto.", "resolution": "Retain both raw vectors and findings; no averaged replacement or cosmetic round."}, "freeze_integrity": {"opus": "Verified persisted checks/opus-r4-freeze.json bytes against publisher hash. Quality vectors, observations, totals, brand vectors/observations/N/A exclusions all unchanged. Final brand records add mean_exact_fraction only (all32); raw full-vector digest therefore differs if derived metadata is included.", "opus_frozen_file_sha256": "8fe9a11f471f7fc4efe0557de120ad6313a26a5748472248ec4ee1ab1dc85a97", "sol": "Full files-array digest reproduces050708ca86dab5500f6bf13595fa14bf7ff4b006d6c08a40a6689ae66c8958e0."}, "drift": "Opus raw mean rises0.09375; Sol raw mean falls0.1. Both disclose variance on unchanged images. Never use variance-adjusted estimates as progression scores.", "remaining_findings": ["Phone contacts row density/alignment, clipped search hint and repeated count.", "Contact-editor photo helper placement and disclosure spacing.", "Phone bulk toolbar wrap; optional navigation-label consistency."], "limitations": ["Everyday-user initial views only; full behavior/roles/states/all named themes/assistive-tech/competitive gates remain untested.", "Opus live supplement uses a different browser/DPR and does not replace scored originals.", "Current-head whole-repository hostedCI and security review remain pending."], "gemini": "Unavailable: quota reached; no score", "dox_pass": "Evidence records and existing exporter only. Owning AGENTS and parent indexes intentionally unchanged: ownership, structure and progression contracts are unchanged."}</t>
         </is>
       </c>
     </row>
@@ -44679,7 +44679,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending advisory</t>
+          <t xml:space="preserve">Unavailable: quota reached; no score</t>
         </is>
       </c>
     </row>

</xml_diff>